<commit_message>
Updated BRA_grids model - 2025-09-17 19:28
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/SuppXLS/Scen_Base_VS.xlsx
+++ b/VerveStacks_BRA_grids/SuppXLS/Scen_Base_VS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7CD00E1E-693A-4AFE-8ABA-4CBE80763281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3DA0A47C-4E40-4ACB-B8C9-4329B9D3A481}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6426,7 +6426,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D91C6E8F-BFE1-4014-8B4A-4FFF5489E0D9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C6288E6-4B8F-490E-AD6E-2D7744AB68E3}">
   <dimension ref="B2:AE915"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA_grids model - 2025-09-22 21:00
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/SuppXLS/Scen_Base_VS.xlsx
+++ b/VerveStacks_BRA_grids/SuppXLS/Scen_Base_VS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E8E802E2-D34D-43E4-BE2A-9B44A0433A22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E8EAB86B-A2BF-4206-9393-3A40426F52B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7380,7 +7380,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DA4C410-50EA-4BC7-B670-8767800D9136}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C5C3A6E-D760-4A16-A548-2F8DBA06B6B8}">
   <dimension ref="B2:AE1072"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated BRA_grids model - 2025-09-22 21:08
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/SuppXLS/Scen_Base_VS.xlsx
+++ b/VerveStacks_BRA_grids/SuppXLS/Scen_Base_VS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E8EAB86B-A2BF-4206-9393-3A40426F52B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{651A25BA-9CE9-4379-B9B0-C9C8A0A5201E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7380,7 +7380,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C5C3A6E-D760-4A16-A548-2F8DBA06B6B8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67B455FA-F6A1-4D04-8E0A-5F4AAAA7C4E3}">
   <dimension ref="B2:AE1072"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>